<commit_message>
werkend krijgen en eerste test run
</commit_message>
<xml_diff>
--- a/gate_assignment_results.xlsx
+++ b/gate_assignment_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,7 +443,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>x_ijh[F3,F4,G3]</t>
+          <t>x_ijh[F8,F51,Fedex 01]</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -453,7 +453,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>x_ijh[F0,F3,G3]</t>
+          <t>x_ijh[F0,F8,Fedex 01]</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -463,7 +463,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>x_ijh[F2,F4,G2]</t>
+          <t>x_ijh[F9,F27,Fedex 14]</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -473,7 +473,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>x_ijh[F0,F2,G2]</t>
+          <t>x_ijh[F27,F51,Fedex 14]</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -483,7 +483,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>x_ijh[F1,F4,G1]</t>
+          <t>x_ijh[F0,F9,Fedex 14]</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -493,7 +493,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>x_ijh[F0,F1,G1]</t>
+          <t>x_ijh[F28,F51,Terminal 1, Gate 206]</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -503,7 +503,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>y_igamma[F1,1]</t>
+          <t>x_ijh[F0,F28,Terminal 1, Gate 206]</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -513,7 +513,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>y_igamma[F2,3]</t>
+          <t>x_ijh[F6,F15,Terminal 1, Gate 230]</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -523,10 +523,1200 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>y_igamma[F3,3]</t>
+          <t>x_ijh[F7,F6,Terminal 1, Gate 230]</t>
         </is>
       </c>
       <c r="B10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>x_ijh[F15,F51,Terminal 1, Gate 230]</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>x_ijh[F19,F7,Terminal 1, Gate 230]</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>x_ijh[F21,F22,Terminal 1, Gate 230]</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>x_ijh[F22,F19,Terminal 1, Gate 230]</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F21,Terminal 1, Gate 230]</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>x_ijh[F45,F51,Cargo 501]</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F45,Cargo 501]</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>x_ijh[F43,F51,Cargo 505]</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F43,Cargo 505]</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>x_ijh[F31,F35,Terminal 1, Gate 129]</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>x_ijh[F35,F51,Terminal 1, Gate 129]</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F31,Terminal 1, Gate 129]</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>x_ijh[F12,F51,Fbo Stand Yl06]</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F12,Fbo Stand Yl06]</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>x_ijh[F2,F51,Fbo Stand Yl07]</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F2,Fbo Stand Yl07]</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>x_ijh[F13,F51,Fbo Stand Yl08]</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F13,Fbo Stand Yl08]</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>x_ijh[F40,F51,Fbo Stand Yt06]</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F40,Fbo Stand Yt06]</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>x_ijh[F37,F51,Fbo Stand Yt08]</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F37,Fbo Stand Yt08]</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>x_ijh[F23,F51,Fbo Stand Yt09]</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>x_ijh[F32,F23,Fbo Stand Yt09]</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F32,Fbo Stand Yt09]</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>x_ijh[F1,F11,Fbo Stand Yt10]</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>x_ijh[F11,F18,Fbo Stand Yt10]</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>x_ijh[F18,F51,Fbo Stand Yt10]</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F1,Fbo Stand Yt10]</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>x_ijh[F48,F51,Fbo Stand Yt12]</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F48,Fbo Stand Yt12]</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>x_ijh[F17,F51,Fbo Stand Yt15]</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F17,Fbo Stand Yt15]</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>x_ijh[F47,F51,Fbo Stand Yt16]</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F47,Fbo Stand Yt16]</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>x_ijh[F24,F41,Fbo Stand Yt17]</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>x_ijh[F41,F51,Fbo Stand Yt17]</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F24,Fbo Stand Yt17]</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>x_ijh[F26,F30,Terminal 1, Gate 205]</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>x_ijh[F30,F51,Terminal 1, Gate 205]</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F26,Terminal 1, Gate 205]</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>x_ijh[F44,F51,Terminal 2, Gate 254]</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F44,Terminal 2, Gate 254]</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>x_ijh[F20,F51,Terminal 2, Gate 255]</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>x_ijh[F39,F20,Terminal 2, Gate 255]</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F39,Terminal 2, Gate 255]</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>x_ijh[F50,F51,Terminal 1, Gate 219]</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F50,Terminal 1, Gate 219]</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>x_ijh[F25,F51,Terminal 2, Gate 254R]</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F25,Terminal 2, Gate 254R]</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>x_ijh[F4,F51,Terminal 2, Gate 255L]</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F4,Terminal 2, Gate 255L]</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>x_ijh[F49,F51,Terminal 1, Gate 128]</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F49,Terminal 1, Gate 128]</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>x_ijh[F10,F51,Terminal 1, Gate 229]</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>x_ijh[F16,F10,Terminal 1, Gate 229]</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>x_ijh[F29,F16,Terminal 1, Gate 229]</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>x_ijh[F36,F29,Terminal 1, Gate 229]</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>x_ijh[F46,F36,Terminal 1, Gate 229]</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F46,Terminal 1, Gate 229]</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>x_ijh[F3,F42,Terminal 1, Gate 231]</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>x_ijh[F5,F34,Terminal 1, Gate 231]</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>x_ijh[F33,F51,Terminal 1, Gate 231]</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>x_ijh[F34,F38,Terminal 1, Gate 231]</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>x_ijh[F38,F33,Terminal 1, Gate 231]</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>x_ijh[F42,F5,Terminal 1, Gate 231]</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F3,Terminal 1, Gate 231]</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>x_ijh[F14,F51,Terminal 1, Gate 218]</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>x_ijh[F0,F14,Terminal 1, Gate 218]</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>y_igamma[F1,2]</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>y_igamma[F2,2]</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>y_igamma[F3,1]</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>y_igamma[F4,1]</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>y_igamma[F5,1]</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>y_igamma[F6,1]</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>y_igamma[F7,1]</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>y_igamma[F8,2]</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>y_igamma[F9,2]</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>y_igamma[F10,1]</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>y_igamma[F11,2]</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>y_igamma[F12,2]</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>y_igamma[F13,2]</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>y_igamma[F14,1]</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>y_igamma[F15,1]</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>y_igamma[F16,1]</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>y_igamma[F17,2]</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>y_igamma[F18,2]</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>y_igamma[F19,1]</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>y_igamma[F20,1]</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>y_igamma[F21,1]</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>y_igamma[F22,1]</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>y_igamma[F23,2]</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>y_igamma[F24,2]</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>y_igamma[F25,1]</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>y_igamma[F26,1]</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>y_igamma[F27,2]</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>y_igamma[F28,1]</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>y_igamma[F29,1]</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>y_igamma[F30,1]</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>y_igamma[F31,2]</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>y_igamma[F32,2]</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>y_igamma[F33,1]</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>y_igamma[F34,1]</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>y_igamma[F35,2]</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>y_igamma[F36,1]</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>y_igamma[F37,2]</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>y_igamma[F38,1]</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>y_igamma[F39,1]</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>y_igamma[F40,2]</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>y_igamma[F41,2]</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>y_igamma[F42,1]</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>y_igamma[F43,1]</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>y_igamma[F44,1]</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>y_igamma[F45,1]</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>y_igamma[F46,1]</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>y_igamma[F47,2]</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>y_igamma[F48,2]</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>y_igamma[F49,2]</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>y_igamma[F50,1]</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>